<commit_message>
função 00 juntei 100 redes e agora tenho que fazer os ensembles
</commit_message>
<xml_diff>
--- a/fuction_ensemble/redes-ensemble-s/Teste03/content/results/metrics_19_9.xlsx
+++ b/fuction_ensemble/redes-ensemble-s/Teste03/content/results/metrics_19_9.xlsx
@@ -513,386 +513,386 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_11</t>
+          <t>model_19_9_0</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9850586968909466</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7210179974427638</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9733183331927504</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8802493293208391</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9638617350973946</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G2" t="n">
-        <v>0.09991256268861463</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H2" t="n">
-        <v>1.865553935694241</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2212452514354178</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3079644141927776</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2646048008127673</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L2" t="n">
-        <v>1.323400365239595</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M2" t="n">
-        <v>0.3160894852547529</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N2" t="n">
-        <v>1.007031201463084</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3295460690374858</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P2" t="n">
-        <v>154.6069196971901</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q2" t="n">
-        <v>246.0226065623051</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_12</t>
+          <t>model_19_9_22</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9843020402774937</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C3" t="n">
-        <v>0.720986125270213</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9716691618546338</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8662367759823041</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9604671020798632</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1049723289468578</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H3" t="n">
-        <v>1.865767065058847</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2349202339617176</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J3" t="n">
-        <v>0.3440006865223819</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K3" t="n">
-        <v>0.2894603437077324</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L3" t="n">
-        <v>1.364925530413878</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M3" t="n">
-        <v>0.3239943347450042</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N3" t="n">
-        <v>1.007387275163532</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3377874443358315</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P3" t="n">
-        <v>154.5081169947904</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q3" t="n">
-        <v>245.9238038599055</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_10</t>
+          <t>model_19_9_21</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9857442123366187</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7209013011835362</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9749490735864221</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8948160292977649</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9673432555368626</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G4" t="n">
-        <v>0.09532851774689757</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H4" t="n">
-        <v>1.866334284117033</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2077230989016126</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J4" t="n">
-        <v>0.2705030354825491</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2391130671920808</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L4" t="n">
-        <v>1.279006416855804</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3087531663755007</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N4" t="n">
-        <v>1.006708605959238</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3218974278752701</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P4" t="n">
-        <v>154.7008525425013</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q4" t="n">
-        <v>246.1165394076164</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_13</t>
+          <t>model_19_9_20</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9835067272443911</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7208458146106437</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9700333002883457</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8528897248684435</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9571968267087687</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1102905908612941</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H5" t="n">
-        <v>1.866705323085458</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2484848514258942</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3783254778088864</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K5" t="n">
-        <v>0.3134053384523185</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L5" t="n">
-        <v>1.402619906239042</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3321002722993374</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N5" t="n">
-        <v>1.007761540120287</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O5" t="n">
-        <v>0.3462384684334566</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P5" t="n">
-        <v>154.409273322672</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q5" t="n">
-        <v>245.8249601877871</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_14</t>
+          <t>model_19_9_19</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.982697630835882</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7206288722200178</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9684351947308691</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8402789954948077</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9540772767177664</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1157010222705415</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H6" t="n">
-        <v>1.868156017850501</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2617363948335258</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4107566605494039</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K6" t="n">
-        <v>0.3362467201904643</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L6" t="n">
-        <v>1.436802697514414</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3401485297197997</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N6" t="n">
-        <v>1.00814229137135</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O6" t="n">
-        <v>0.3546293568344976</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P6" t="n">
-        <v>154.3134916185879</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q6" t="n">
-        <v>245.729178483703</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_9</t>
+          <t>model_19_9_18</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9863167234696129</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7205846276108299</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9765218283449422</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9097746512203889</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9708607721439736</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G7" t="n">
-        <v>0.09150013316439386</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H7" t="n">
-        <v>1.868451881755869</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1946817651457894</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2320337458209104</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2133577692083889</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L7" t="n">
-        <v>1.231021360970968</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M7" t="n">
-        <v>0.3024898893589567</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N7" t="n">
-        <v>1.006439188955476</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3153675101893612</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P7" t="n">
-        <v>154.7828297027063</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q7" t="n">
-        <v>246.1985165678213</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_15</t>
+          <t>model_19_9_17</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9818934200546353</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7203598859972304</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9668932283292814</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8284427947437927</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9511255643992187</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1210787834677882</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H8" t="n">
-        <v>1.869954729960848</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2745224305294504</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J8" t="n">
-        <v>0.4411959775893943</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K8" t="n">
-        <v>0.3578591925161511</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L8" t="n">
-        <v>1.467773922793117</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3479637674640683</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N8" t="n">
-        <v>1.008520743503701</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O8" t="n">
-        <v>0.362777305429312</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P8" t="n">
-        <v>154.2226276844429</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q8" t="n">
-        <v>245.6383145495579</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="9">
@@ -902,547 +902,547 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9811078942553135</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7200578771261772</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9654202575940112</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8173976339466456</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9483518094058899</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1263315981048667</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H9" t="n">
-        <v>1.871974264672203</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2867363519098531</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J9" t="n">
-        <v>0.4696009665156933</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K9" t="n">
-        <v>0.3781686592127732</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L9" t="n">
-        <v>1.495806281530666</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M9" t="n">
-        <v>0.3554315659938868</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N9" t="n">
-        <v>1.008890402703382</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O9" t="n">
-        <v>0.370563023603019</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P9" t="n">
-        <v>154.1376901959597</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q9" t="n">
-        <v>245.5533770610747</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_8</t>
+          <t>model_19_9_15</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9867234874491739</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C10" t="n">
-        <v>0.7200031321901419</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9779899964953158</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9249015695351914</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F10" t="n">
-        <v>0.974348628895075</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G10" t="n">
-        <v>0.08878010056009338</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H10" t="n">
-        <v>1.872340344311549</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1825076669559925</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1931316460586345</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1878196410393711</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L10" t="n">
-        <v>1.178344285182996</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2979598975702827</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N10" t="n">
-        <v>1.006247770612154</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O10" t="n">
-        <v>0.3106446672718676</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P10" t="n">
-        <v>154.8431854937766</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q10" t="n">
-        <v>246.2588723588916</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_17</t>
+          <t>model_19_9_14</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.9803507196832072</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7197374242720274</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9640249494396693</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8071379618377348</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F11" t="n">
-        <v>0.945759975425183</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1313948279550097</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H11" t="n">
-        <v>1.874117134383454</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2983062926360972</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J11" t="n">
-        <v>0.4959859035929647</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K11" t="n">
-        <v>0.3971460981145309</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L11" t="n">
-        <v>1.521162846662782</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M11" t="n">
-        <v>0.3624842451128182</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N11" t="n">
-        <v>1.009246720149079</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O11" t="n">
-        <v>0.3779159498731018</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P11" t="n">
-        <v>154.0590970695586</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q11" t="n">
-        <v>245.4747839346736</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_18</t>
+          <t>model_19_9_13</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.979628666934124</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C12" t="n">
-        <v>0.719409664384788</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9627124085602662</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7976477746134317</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F12" t="n">
-        <v>0.9433501408512048</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1362231980128766</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H12" t="n">
-        <v>1.876308866258619</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3091899244189475</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5203919460187534</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K12" t="n">
-        <v>0.4147909352188505</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L12" t="n">
-        <v>1.544077854339795</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3690842695278093</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N12" t="n">
-        <v>1.009586509678059</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O12" t="n">
-        <v>0.384796950991373</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P12" t="n">
-        <v>153.9869211532424</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q12" t="n">
-        <v>245.4026080183574</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_19</t>
+          <t>model_19_9_23</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.978945782056741</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C13" t="n">
-        <v>0.7190825651079283</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9614848533864704</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7888976172820026</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F13" t="n">
-        <v>0.9411183891032593</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1407896523323327</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H13" t="n">
-        <v>1.878496180629133</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3193688519589434</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5428948435923963</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K13" t="n">
-        <v>0.4311318477756698</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L13" t="n">
-        <v>1.564786378658034</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M13" t="n">
-        <v>0.375219472219037</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N13" t="n">
-        <v>1.009907867267416</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O13" t="n">
-        <v>0.3911933419627867</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P13" t="n">
-        <v>153.9209766598335</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q13" t="n">
-        <v>245.3366635249485</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_7</t>
+          <t>model_19_9_12</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.9868984321807623</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C14" t="n">
-        <v>0.7190747812612519</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9793000164612712</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9398966834705936</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F14" t="n">
-        <v>0.9777237828550907</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G14" t="n">
-        <v>0.08761024433441525</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H14" t="n">
-        <v>1.8785482312477</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I14" t="n">
-        <v>0.171644938669675</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1545685093957708</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1631067240327229</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L14" t="n">
-        <v>1.120625250094653</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2959902774322414</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N14" t="n">
-        <v>1.006165443679641</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O14" t="n">
-        <v>0.3085911963268741</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P14" t="n">
-        <v>154.8697146868409</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q14" t="n">
-        <v>246.285401551956</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_20</t>
+          <t>model_19_9_10</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.9783044061813996</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C15" t="n">
-        <v>0.7187622232426423</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9603423194567582</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E15" t="n">
-        <v>0.780853402792072</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F15" t="n">
-        <v>0.9390587198259862</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1450785357640052</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H15" t="n">
-        <v>1.880638308157339</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3288427805698795</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5635822584434568</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K15" t="n">
-        <v>0.4462127704575374</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L15" t="n">
-        <v>1.583484571243272</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M15" t="n">
-        <v>0.3808917638437528</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N15" t="n">
-        <v>1.010209691208753</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O15" t="n">
-        <v>0.3971071147852291</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P15" t="n">
-        <v>153.8609601144586</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q15" t="n">
-        <v>245.2766469795737</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_21</t>
+          <t>model_19_9_9</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.9777056388136918</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C16" t="n">
-        <v>0.7184528676250079</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9592838406156489</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E16" t="n">
-        <v>0.7734785049356938</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9371642604991791</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1490824959089372</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H16" t="n">
-        <v>1.882706970596912</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I16" t="n">
-        <v>0.3376197216445154</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5825483826846828</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K16" t="n">
-        <v>0.4600840239382639</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L16" t="n">
-        <v>1.600353586114625</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M16" t="n">
-        <v>0.3861120250768386</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N16" t="n">
-        <v>1.010491464087675</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O16" t="n">
-        <v>0.4025496133464377</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P16" t="n">
-        <v>153.8065109248671</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q16" t="n">
-        <v>245.2221977899822</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_22</t>
+          <t>model_19_9_8</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.9771491934441112</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C17" t="n">
-        <v>0.7181574036906784</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9583062937184762</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E17" t="n">
-        <v>0.7667310455448508</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F17" t="n">
-        <v>0.935425777123207</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1528034486575175</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H17" t="n">
-        <v>1.88468273928626</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I17" t="n">
-        <v>0.3457255724002902</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J17" t="n">
-        <v>0.59990091496534</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K17" t="n">
-        <v>0.4728132196717937</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L17" t="n">
-        <v>1.615577952000741</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M17" t="n">
-        <v>0.3909008169056666</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N17" t="n">
-        <v>1.010753320732183</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O17" t="n">
-        <v>0.4075422739575847</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P17" t="n">
-        <v>153.7572056655125</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q17" t="n">
-        <v>245.1728925306276</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_23</t>
+          <t>model_19_9_7</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.9766342437559136</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C18" t="n">
-        <v>0.7178776496160092</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D18" t="n">
-        <v>0.9574065114279743</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7605698969363477</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F18" t="n">
-        <v>0.9338342569531075</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1562469195936205</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H18" t="n">
-        <v>1.886553456071722</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I18" t="n">
-        <v>0.3531865965011211</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J18" t="n">
-        <v>0.6157456239027614</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K18" t="n">
-        <v>0.484466349082783</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L18" t="n">
-        <v>1.629307363664094</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M18" t="n">
-        <v>0.3952808110617318</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N18" t="n">
-        <v>1.010995649997217</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O18" t="n">
-        <v>0.4121087335327114</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P18" t="n">
-        <v>153.7126354103216</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q18" t="n">
-        <v>245.1283222754366</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="19">
@@ -1452,437 +1452,437 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.986760255497919</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C19" t="n">
-        <v>0.7176955508171172</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9803959248425539</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E19" t="n">
-        <v>0.9543690499370948</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9808858987394163</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G19" t="n">
-        <v>0.08853423244883359</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H19" t="n">
-        <v>1.887771151578401</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I19" t="n">
-        <v>0.1625576306270908</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J19" t="n">
-        <v>0.1173497294460495</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K19" t="n">
-        <v>0.1399536743228412</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L19" t="n">
-        <v>1.057498162616016</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2975470256091188</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N19" t="n">
-        <v>1.006230468000979</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O19" t="n">
-        <v>0.3102142184965541</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P19" t="n">
-        <v>154.848731988855</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q19" t="n">
-        <v>246.26441885397</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_24</t>
+          <t>model_19_9_5</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.9761593300622614</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C20" t="n">
-        <v>0.7176146548980009</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D20" t="n">
-        <v>0.9565803973154802</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E20" t="n">
-        <v>0.7549535303179754</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F20" t="n">
-        <v>0.9323801911967057</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G20" t="n">
-        <v>0.159422669649849</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H20" t="n">
-        <v>1.888312102962022</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I20" t="n">
-        <v>0.360036761667094</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J20" t="n">
-        <v>0.6301893096517375</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K20" t="n">
-        <v>0.4951130356594158</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L20" t="n">
-        <v>1.641687063973062</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M20" t="n">
-        <v>0.3992776848884107</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N20" t="n">
-        <v>1.01121913879423</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O20" t="n">
-        <v>0.4162757625528615</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P20" t="n">
-        <v>153.6723926082134</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q20" t="n">
-        <v>245.0880794733285</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_5</t>
+          <t>model_19_9_4</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.9862098391480514</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C21" t="n">
-        <v>0.7157335704931751</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D21" t="n">
-        <v>0.9812228058771263</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9678225085127703</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F21" t="n">
-        <v>0.9837167352033989</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G21" t="n">
-        <v>0.09221486911483243</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H21" t="n">
-        <v>1.90089092303869</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I21" t="n">
-        <v>0.1557011061182306</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J21" t="n">
-        <v>0.08275128865547338</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1192262564264824</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L21" t="n">
-        <v>0.9886921387254725</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M21" t="n">
-        <v>0.3036690124376085</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N21" t="n">
-        <v>1.006489487459741</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O21" t="n">
-        <v>0.3165968309785924</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P21" t="n">
-        <v>154.7672677823926</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q21" t="n">
-        <v>246.1829546475076</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_4</t>
+          <t>model_19_9_3</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.9851270965618283</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C22" t="n">
-        <v>0.7130203056790934</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D22" t="n">
-        <v>0.9817337013206515</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E22" t="n">
-        <v>0.9796321489632606</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F22" t="n">
-        <v>0.9860799979756126</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G22" t="n">
-        <v>0.09945517377447757</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H22" t="n">
-        <v>1.91903453734389</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1514647444367619</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J22" t="n">
-        <v>0.05238027709841263</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K22" t="n">
-        <v>0.1019224186026366</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L22" t="n">
-        <v>0.914159276868971</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M22" t="n">
-        <v>0.315365143562946</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N22" t="n">
-        <v>1.006999013382669</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O22" t="n">
-        <v>0.3287908906202648</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P22" t="n">
-        <v>154.6160965023185</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q22" t="n">
-        <v>246.0317833674335</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_3</t>
+          <t>model_19_9_2</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.9833644011222131</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C23" t="n">
-        <v>0.7093404468858818</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D23" t="n">
-        <v>0.9818856934092327</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E23" t="n">
-        <v>0.98901451085</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F23" t="n">
-        <v>0.987813734985993</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1112423262956506</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H23" t="n">
-        <v>1.943641770038287</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1502044210807563</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J23" t="n">
-        <v>0.02825153054687298</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K23" t="n">
-        <v>0.08922797581381464</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L23" t="n">
-        <v>0.8346218686027407</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M23" t="n">
-        <v>0.3335300980356204</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N23" t="n">
-        <v>1.007828517118958</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O23" t="n">
-        <v>0.3477291648114805</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P23" t="n">
-        <v>154.3920886748651</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q23" t="n">
-        <v>245.8077755399802</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_2</t>
+          <t>model_19_9_1</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.9807331389949939</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C24" t="n">
-        <v>0.704422555148253</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9816102040175444</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9949599547131333</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F24" t="n">
-        <v>0.9887018523183791</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1288375882562135</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H24" t="n">
-        <v>1.976527734732621</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I24" t="n">
-        <v>0.1524887881022086</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J24" t="n">
-        <v>0.01296155241112225</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K24" t="n">
-        <v>0.08272517025666545</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L24" t="n">
-        <v>0.7519948306703753</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M24" t="n">
-        <v>0.3589395328689965</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N24" t="n">
-        <v>1.009066758120003</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O24" t="n">
-        <v>0.3742203318904948</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P24" t="n">
-        <v>154.0984053471997</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q24" t="n">
-        <v>245.5140922123148</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_1</t>
+          <t>model_19_9_11</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.9769723929580898</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C25" t="n">
-        <v>0.6979432903980837</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D25" t="n">
-        <v>0.9807096243802936</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E25" t="n">
-        <v>0.996084797306776</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F25" t="n">
-        <v>0.9883894424931269</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G25" t="n">
-        <v>0.153985714321634</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H25" t="n">
-        <v>2.019854607951274</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I25" t="n">
-        <v>0.1599564238282885</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J25" t="n">
-        <v>0.01006877954859363</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K25" t="n">
-        <v>0.08501263867291647</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L25" t="n">
-        <v>0.677296651763879</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M25" t="n">
-        <v>0.3924101353451948</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N25" t="n">
-        <v>1.010836520960899</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O25" t="n">
-        <v>0.4091158472078034</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P25" t="n">
-        <v>153.7417908900332</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q25" t="n">
-        <v>245.1574777551482</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>model_19_9_0</t>
+          <t>model_19_9_24</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.9716999889318237</v>
+        <v>0.9933671815352429</v>
       </c>
       <c r="C26" t="n">
-        <v>0.6895644302308013</v>
+        <v>0.6021233998827213</v>
       </c>
       <c r="D26" t="n">
-        <v>0.9786881101842958</v>
+        <v>0.9995841116269548</v>
       </c>
       <c r="E26" t="n">
-        <v>0.9903351261551905</v>
+        <v>0.9999992911975398</v>
       </c>
       <c r="F26" t="n">
-        <v>0.9862350420807231</v>
+        <v>0.9999330175453384</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1892423043224635</v>
+        <v>0.003937527563518465</v>
       </c>
       <c r="H26" t="n">
-        <v>2.075884084470995</v>
+        <v>0.2361967372038093</v>
       </c>
       <c r="I26" t="n">
-        <v>0.176718885476759</v>
+        <v>9.50105965787351e-05</v>
       </c>
       <c r="J26" t="n">
-        <v>0.02485528636276639</v>
+        <v>8.082987839984312e-07</v>
       </c>
       <c r="K26" t="n">
-        <v>0.100787183840799</v>
+        <v>4.790944768442717e-05</v>
       </c>
       <c r="L26" t="n">
-        <v>0.6119454174932583</v>
+        <v>0.01203164107885965</v>
       </c>
       <c r="M26" t="n">
-        <v>0.4350198895711131</v>
+        <v>0.06274972162104359</v>
       </c>
       <c r="N26" t="n">
-        <v>1.013317652267377</v>
+        <v>1.008378297008114</v>
       </c>
       <c r="O26" t="n">
-        <v>0.4535395868854701</v>
+        <v>0.0654211071802823</v>
       </c>
       <c r="P26" t="n">
-        <v>153.329454103147</v>
+        <v>97.07440454919247</v>
       </c>
       <c r="Q26" t="n">
-        <v>244.745140968262</v>
+        <v>149.4860650185251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>